<commit_message>
Enhance PAFFP Formatter: Update descriptions, add amount input, and include System Upload template
- Updated meta description for clarity on file creation.
- Improved instructional text for file uploads and formats.
- Added input field for specifying an amount when masterlist lacks one.
- Adjusted API call to include amount in request.
- Updated Vercel configuration to include new System Uploading Template.
- Introduced System Uploading Template.xlsx for consistent file generation.
</commit_message>
<xml_diff>
--- a/STUB FORMAT.xlsx
+++ b/STUB FORMAT.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.1769" customWidth="1" min="1" max="1"/>
@@ -547,106 +547,14 @@
       <c r="F2" s="3" t="n"/>
       <c r="G2" s="3" t="n"/>
     </row>
-    <row r="3" ht="20.75" customHeight="1">
-      <c r="A3" s="4" t="n"/>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-    </row>
-    <row r="4" ht="14.5" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Certified true and correct:</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Recommending Approval:</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Approved for Payment:</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>Payment Received by Payee:</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="23.75" customHeight="1">
-      <c r="A5" s="7" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="7" t="n"/>
-    </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>DANILO P. DAGUIO, Ph.D.,CESO IV</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>ATTY. JENNILYN M. DAWAYAN, CESO III</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="7" t="n"/>
-    </row>
-    <row r="7" ht="31.25" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>RSBSA/Personnel who handles the list of beneficiaries</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Regional Technical Director</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>Regional Executive Director/Head of Agency</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>Special Disbursing Officer</t>
-        </is>
-      </c>
-    </row>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C4:D4"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>